<commit_message>
fixed spain country map that was overwritten with madrid map and saving R data
</commit_message>
<xml_diff>
--- a/data/spain_datacenters_v2.xlsx
+++ b/data/spain_datacenters_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bca0b3a3594cbf72/Desktop/Learning/Grad_School/geospatial/GeoFinal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{52B6B1E7-5C99-4850-8BA2-1A4FC0C1EA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{52B6B1E7-5C99-4850-8BA2-1A4FC0C1EA57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B96AE75-3EA8-49B2-B2AD-443DF20725FD}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1615,7 +1615,7 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1625,34 +1625,34 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1955,6 +1955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I209"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2025,7 +2026,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
         <v>256</v>
       </c>
@@ -2048,7 +2049,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
         <v>141</v>
       </c>
@@ -2073,7 +2074,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>141</v>
       </c>
@@ -2098,7 +2099,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8" t="s">
         <v>141</v>
       </c>
@@ -2123,7 +2124,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8" t="s">
         <v>279</v>
       </c>
@@ -2173,7 +2174,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>408</v>
       </c>
@@ -2194,7 +2195,7 @@
       <c r="H9" s="9"/>
       <c r="I9" s="11"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="8" t="s">
         <v>408</v>
       </c>
@@ -2263,7 +2264,7 @@
       <c r="H12" s="9"/>
       <c r="I12" s="11"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8" t="s">
         <v>408</v>
       </c>
@@ -2286,7 +2287,7 @@
       <c r="H13" s="9"/>
       <c r="I13" s="11"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="8" t="s">
         <v>408</v>
       </c>
@@ -2330,7 +2331,7 @@
       <c r="H15" s="9"/>
       <c r="I15" s="11"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="8" t="s">
         <v>408</v>
       </c>
@@ -2378,7 +2379,7 @@
       <c r="H17" s="9"/>
       <c r="I17" s="11"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="8" t="s">
         <v>408</v>
       </c>
@@ -2399,7 +2400,7 @@
       <c r="H18" s="9"/>
       <c r="I18" s="11"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
         <v>408</v>
       </c>
@@ -2420,7 +2421,7 @@
       <c r="H19" s="9"/>
       <c r="I19" s="11"/>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="8" t="s">
         <v>408</v>
       </c>
@@ -2489,7 +2490,7 @@
       <c r="H22" s="9"/>
       <c r="I22" s="11"/>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="8" t="s">
         <v>408</v>
       </c>
@@ -2537,7 +2538,7 @@
       <c r="H24" s="9"/>
       <c r="I24" s="11"/>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
         <v>408</v>
       </c>
@@ -2556,7 +2557,7 @@
       <c r="H25" s="9"/>
       <c r="I25" s="11"/>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="8" t="s">
         <v>408</v>
       </c>
@@ -2577,7 +2578,7 @@
       <c r="H26" s="9"/>
       <c r="I26" s="11"/>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8" t="s">
         <v>408</v>
       </c>
@@ -2598,7 +2599,7 @@
       <c r="H27" s="9"/>
       <c r="I27" s="11"/>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8" t="s">
         <v>408</v>
       </c>
@@ -2619,7 +2620,7 @@
       <c r="H28" s="9"/>
       <c r="I28" s="11"/>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
         <v>408</v>
       </c>
@@ -2640,7 +2641,7 @@
       <c r="H29" s="9"/>
       <c r="I29" s="11"/>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="8" t="s">
         <v>408</v>
       </c>
@@ -2711,7 +2712,7 @@
       <c r="H32" s="9"/>
       <c r="I32" s="11"/>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="8" t="s">
         <v>408</v>
       </c>
@@ -2755,7 +2756,7 @@
       <c r="H34" s="9"/>
       <c r="I34" s="11"/>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="8" t="s">
         <v>408</v>
       </c>
@@ -2776,7 +2777,7 @@
       <c r="H35" s="9"/>
       <c r="I35" s="11"/>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="8" t="s">
         <v>408</v>
       </c>
@@ -2797,7 +2798,7 @@
       <c r="H36" s="9"/>
       <c r="I36" s="11"/>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="8" t="s">
         <v>408</v>
       </c>
@@ -2818,7 +2819,7 @@
       <c r="H37" s="9"/>
       <c r="I37" s="11"/>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="8" t="s">
         <v>408</v>
       </c>
@@ -2839,7 +2840,7 @@
       <c r="H38" s="9"/>
       <c r="I38" s="11"/>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="8" t="s">
         <v>408</v>
       </c>
@@ -2860,7 +2861,7 @@
       <c r="H39" s="9"/>
       <c r="I39" s="11"/>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="8" t="s">
         <v>408</v>
       </c>
@@ -2881,7 +2882,7 @@
       <c r="H40" s="9"/>
       <c r="I40" s="11"/>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="8" t="s">
         <v>408</v>
       </c>
@@ -2902,7 +2903,7 @@
       <c r="H41" s="9"/>
       <c r="I41" s="11"/>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="8" t="s">
         <v>408</v>
       </c>
@@ -2923,7 +2924,7 @@
       <c r="H42" s="9"/>
       <c r="I42" s="11"/>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="8" t="s">
         <v>78</v>
       </c>
@@ -2946,7 +2947,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="8" t="s">
         <v>78</v>
       </c>
@@ -3077,7 +3078,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="8" t="s">
         <v>78</v>
       </c>
@@ -3100,7 +3101,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="8" t="s">
         <v>78</v>
       </c>
@@ -3123,7 +3124,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="8" t="s">
         <v>78</v>
       </c>
@@ -3146,7 +3147,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="8" t="s">
         <v>78</v>
       </c>
@@ -3196,7 +3197,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="8" t="s">
         <v>150</v>
       </c>
@@ -3221,7 +3222,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="8" t="s">
         <v>150</v>
       </c>
@@ -3244,7 +3245,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="8" t="s">
         <v>150</v>
       </c>
@@ -3296,7 +3297,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="8" t="s">
         <v>176</v>
       </c>
@@ -3379,7 +3380,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="8" t="s">
         <v>68</v>
       </c>
@@ -3404,7 +3405,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="8" t="s">
         <v>264</v>
       </c>
@@ -3452,7 +3453,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="8" t="s">
         <v>160</v>
       </c>
@@ -3479,7 +3480,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="8" t="s">
         <v>160</v>
       </c>
@@ -3504,7 +3505,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="8" t="s">
         <v>247</v>
       </c>
@@ -3531,7 +3532,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="8" t="s">
         <v>283</v>
       </c>
@@ -3554,7 +3555,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="8" t="s">
         <v>287</v>
       </c>
@@ -3577,7 +3578,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="8" t="s">
         <v>252</v>
       </c>
@@ -3600,7 +3601,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="8" t="s">
         <v>36</v>
       </c>
@@ -3627,7 +3628,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="8" t="s">
         <v>291</v>
       </c>
@@ -3650,7 +3651,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="8" t="s">
         <v>295</v>
       </c>
@@ -3671,7 +3672,7 @@
       <c r="H72" s="9"/>
       <c r="I72" s="11"/>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="8" t="s">
         <v>295</v>
       </c>
@@ -3692,7 +3693,7 @@
       <c r="H73" s="9"/>
       <c r="I73" s="11"/>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="8" t="s">
         <v>295</v>
       </c>
@@ -3713,7 +3714,7 @@
       <c r="H74" s="9"/>
       <c r="I74" s="11"/>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="8" t="s">
         <v>295</v>
       </c>
@@ -3784,7 +3785,7 @@
       <c r="H77" s="9"/>
       <c r="I77" s="11"/>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="8" t="s">
         <v>295</v>
       </c>
@@ -3805,7 +3806,7 @@
       <c r="H78" s="9"/>
       <c r="I78" s="11"/>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="8" t="s">
         <v>295</v>
       </c>
@@ -3853,7 +3854,7 @@
       <c r="H80" s="9"/>
       <c r="I80" s="11"/>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="8" t="s">
         <v>295</v>
       </c>
@@ -3874,7 +3875,7 @@
       <c r="H81" s="9"/>
       <c r="I81" s="11"/>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="8" t="s">
         <v>295</v>
       </c>
@@ -3893,7 +3894,7 @@
       <c r="H82" s="9"/>
       <c r="I82" s="11"/>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="8" t="s">
         <v>295</v>
       </c>
@@ -3939,7 +3940,7 @@
       <c r="H84" s="9"/>
       <c r="I84" s="11"/>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="8" t="s">
         <v>295</v>
       </c>
@@ -4008,7 +4009,7 @@
       <c r="H87" s="9"/>
       <c r="I87" s="11"/>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="8" t="s">
         <v>295</v>
       </c>
@@ -4029,7 +4030,7 @@
       <c r="H88" s="9"/>
       <c r="I88" s="11"/>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="8" t="s">
         <v>295</v>
       </c>
@@ -4050,7 +4051,7 @@
       <c r="H89" s="9"/>
       <c r="I89" s="11"/>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="8" t="s">
         <v>295</v>
       </c>
@@ -4073,7 +4074,7 @@
       <c r="H90" s="9"/>
       <c r="I90" s="11"/>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="8" t="s">
         <v>295</v>
       </c>
@@ -4096,7 +4097,7 @@
       <c r="H91" s="9"/>
       <c r="I91" s="11"/>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="8" t="s">
         <v>295</v>
       </c>
@@ -4117,7 +4118,7 @@
       <c r="H92" s="9"/>
       <c r="I92" s="11"/>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="8" t="s">
         <v>295</v>
       </c>
@@ -4138,7 +4139,7 @@
       <c r="H93" s="9"/>
       <c r="I93" s="11"/>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="8" t="s">
         <v>295</v>
       </c>
@@ -4159,7 +4160,7 @@
       <c r="H94" s="9"/>
       <c r="I94" s="11"/>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="8" t="s">
         <v>295</v>
       </c>
@@ -4180,7 +4181,7 @@
       <c r="H95" s="9"/>
       <c r="I95" s="11"/>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="8" t="s">
         <v>295</v>
       </c>
@@ -4201,7 +4202,7 @@
       <c r="H96" s="9"/>
       <c r="I96" s="11"/>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="8" t="s">
         <v>295</v>
       </c>
@@ -4360,7 +4361,7 @@
       <c r="H103" s="9"/>
       <c r="I103" s="11"/>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="8" t="s">
         <v>295</v>
       </c>
@@ -4406,7 +4407,7 @@
       <c r="H105" s="9"/>
       <c r="I105" s="11"/>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="8" t="s">
         <v>295</v>
       </c>
@@ -4427,7 +4428,7 @@
       <c r="H106" s="9"/>
       <c r="I106" s="11"/>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="8" t="s">
         <v>295</v>
       </c>
@@ -4448,7 +4449,7 @@
       <c r="H107" s="9"/>
       <c r="I107" s="11"/>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="8" t="s">
         <v>295</v>
       </c>
@@ -4469,7 +4470,7 @@
       <c r="H108" s="9"/>
       <c r="I108" s="11"/>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="8" t="s">
         <v>295</v>
       </c>
@@ -4490,7 +4491,7 @@
       <c r="H109" s="9"/>
       <c r="I109" s="11"/>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="8" t="s">
         <v>295</v>
       </c>
@@ -4536,7 +4537,7 @@
       <c r="H111" s="9"/>
       <c r="I111" s="11"/>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="8" t="s">
         <v>295</v>
       </c>
@@ -4557,7 +4558,7 @@
       <c r="H112" s="9"/>
       <c r="I112" s="11"/>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="8" t="s">
         <v>295</v>
       </c>
@@ -4578,7 +4579,7 @@
       <c r="H113" s="9"/>
       <c r="I113" s="11"/>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="8" t="s">
         <v>295</v>
       </c>
@@ -4599,7 +4600,7 @@
       <c r="H114" s="9"/>
       <c r="I114" s="11"/>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="8" t="s">
         <v>295</v>
       </c>
@@ -4620,7 +4621,7 @@
       <c r="H115" s="9"/>
       <c r="I115" s="11"/>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="8" t="s">
         <v>295</v>
       </c>
@@ -4641,7 +4642,7 @@
       <c r="H116" s="9"/>
       <c r="I116" s="11"/>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="8" t="s">
         <v>295</v>
       </c>
@@ -4662,7 +4663,7 @@
       <c r="H117" s="9"/>
       <c r="I117" s="11"/>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="8" t="s">
         <v>295</v>
       </c>
@@ -4683,7 +4684,7 @@
       <c r="H118" s="9"/>
       <c r="I118" s="11"/>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="8" t="s">
         <v>295</v>
       </c>
@@ -4702,7 +4703,7 @@
       <c r="H119" s="9"/>
       <c r="I119" s="11"/>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="8" t="s">
         <v>295</v>
       </c>
@@ -4723,7 +4724,7 @@
       <c r="H120" s="9"/>
       <c r="I120" s="11"/>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="8" t="s">
         <v>295</v>
       </c>
@@ -4744,7 +4745,7 @@
       <c r="H121" s="9"/>
       <c r="I121" s="11"/>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="8" t="s">
         <v>295</v>
       </c>
@@ -4765,7 +4766,7 @@
       <c r="H122" s="9"/>
       <c r="I122" s="11"/>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="8" t="s">
         <v>295</v>
       </c>
@@ -4784,7 +4785,7 @@
       <c r="H123" s="9"/>
       <c r="I123" s="11"/>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="8" t="s">
         <v>295</v>
       </c>
@@ -4828,7 +4829,7 @@
       <c r="H125" s="9"/>
       <c r="I125" s="11"/>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="8" t="s">
         <v>295</v>
       </c>
@@ -4949,7 +4950,7 @@
       <c r="H130" s="9"/>
       <c r="I130" s="11"/>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="8" t="s">
         <v>295</v>
       </c>
@@ -4970,7 +4971,7 @@
       <c r="H131" s="9"/>
       <c r="I131" s="11"/>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="8" t="s">
         <v>295</v>
       </c>
@@ -5066,7 +5067,7 @@
       <c r="H135" s="9"/>
       <c r="I135" s="11"/>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="8" t="s">
         <v>295</v>
       </c>
@@ -5087,7 +5088,7 @@
       <c r="H136" s="9"/>
       <c r="I136" s="11"/>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="8" t="s">
         <v>295</v>
       </c>
@@ -5108,7 +5109,7 @@
       <c r="H137" s="9"/>
       <c r="I137" s="11"/>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="8" t="s">
         <v>20</v>
       </c>
@@ -5131,7 +5132,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="8" t="s">
         <v>20</v>
       </c>
@@ -5156,7 +5157,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="8" t="s">
         <v>20</v>
       </c>
@@ -5181,7 +5182,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="8" t="s">
         <v>20</v>
       </c>
@@ -5231,7 +5232,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="8" t="s">
         <v>20</v>
       </c>
@@ -5254,7 +5255,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="8" t="s">
         <v>20</v>
       </c>
@@ -5279,7 +5280,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="8" t="s">
         <v>268</v>
       </c>
@@ -5304,7 +5305,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="8" t="s">
         <v>9</v>
       </c>
@@ -5358,7 +5359,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="8" t="s">
         <v>9</v>
       </c>
@@ -5383,7 +5384,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="8" t="s">
         <v>273</v>
       </c>
@@ -5406,7 +5407,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="8" t="s">
         <v>273</v>
       </c>
@@ -5429,7 +5430,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="8" t="s">
         <v>188</v>
       </c>
@@ -5454,7 +5455,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="8" t="s">
         <v>188</v>
       </c>
@@ -5624,7 +5625,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="8" t="s">
         <v>168</v>
       </c>
@@ -6053,7 +6054,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="8" t="s">
         <v>133</v>
       </c>
@@ -6107,7 +6108,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="8" t="s">
         <v>133</v>
       </c>
@@ -6134,7 +6135,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="8" t="s">
         <v>260</v>
       </c>
@@ -6159,7 +6160,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="179" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="8" t="s">
         <v>183</v>
       </c>
@@ -6186,7 +6187,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="180" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="8" t="s">
         <v>183</v>
       </c>
@@ -6211,7 +6212,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="181" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="8" t="s">
         <v>41</v>
       </c>
@@ -6236,7 +6237,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="182" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="8" t="s">
         <v>41</v>
       </c>
@@ -6259,7 +6260,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="183" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="8" t="s">
         <v>41</v>
       </c>
@@ -6282,7 +6283,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="184" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="8" t="s">
         <v>41</v>
       </c>
@@ -6363,7 +6364,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="187" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" s="8" t="s">
         <v>41</v>
       </c>
@@ -6388,7 +6389,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="188" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="8" t="s">
         <v>41</v>
       </c>
@@ -6411,7 +6412,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="189" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="8" t="s">
         <v>41</v>
       </c>
@@ -6436,7 +6437,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="190" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="8" t="s">
         <v>41</v>
       </c>
@@ -6459,7 +6460,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="191" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="8" t="s">
         <v>41</v>
       </c>
@@ -6507,7 +6508,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="193" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="8" t="s">
         <v>99</v>
       </c>
@@ -6530,7 +6531,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="194" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="8" t="s">
         <v>99</v>
       </c>
@@ -6553,7 +6554,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="195" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="8" t="s">
         <v>99</v>
       </c>
@@ -6576,7 +6577,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="196" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="8" t="s">
         <v>99</v>
       </c>
@@ -6597,7 +6598,7 @@
       <c r="H196" s="9"/>
       <c r="I196" s="11"/>
     </row>
-    <row r="197" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="8" t="s">
         <v>99</v>
       </c>
@@ -6622,7 +6623,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="198" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="8" t="s">
         <v>99</v>
       </c>
@@ -6645,7 +6646,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="199" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="8" t="s">
         <v>99</v>
       </c>
@@ -6668,7 +6669,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="200" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="8" t="s">
         <v>99</v>
       </c>
@@ -6691,7 +6692,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="201" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="8" t="s">
         <v>99</v>
       </c>
@@ -6712,7 +6713,7 @@
       <c r="H201" s="9"/>
       <c r="I201" s="11"/>
     </row>
-    <row r="202" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="8" t="s">
         <v>99</v>
       </c>
@@ -6735,7 +6736,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="203" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="8" t="s">
         <v>99</v>
       </c>
@@ -6758,7 +6759,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="204" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="8" t="s">
         <v>99</v>
       </c>
@@ -6781,7 +6782,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="205" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="8" t="s">
         <v>99</v>
       </c>
@@ -6831,7 +6832,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="207" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="8" t="s">
         <v>99</v>
       </c>
@@ -6881,7 +6882,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="209" spans="1:9" s="1" customFormat="1" ht="12.5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:9" s="1" customFormat="1" ht="12.5" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="16" t="s">
         <v>99</v>
       </c>
@@ -6906,10 +6907,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I209" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I209">
-      <sortCondition ref="A2:A209"/>
-      <sortCondition ref="B2:B209"/>
-    </sortState>
+    <filterColumn colId="6">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
   </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>